<commit_message>
Update schema with echem, chemical terms
</commit_message>
<xml_diff>
--- a/test/data/electrolysis_excel_schema.xlsx
+++ b/test/data/electrolysis_excel_schema.xlsx
@@ -946,7 +946,7 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-hasSubstrate</t>
+          <t>hasNegativeElectrode-echem:hasSubstrate</t>
         </is>
       </c>
       <c r="F15" s="8" t="n"/>
@@ -974,7 +974,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-hasSubstrate</t>
+          <t>hasNegativeElectrode-echem:hasSubstrate</t>
         </is>
       </c>
       <c r="F16" s="4" t="n"/>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-hasSubstrate-hasCoating</t>
+          <t>hasNegativeElectrode-echem:hasSubstrate-hasCoating</t>
         </is>
       </c>
       <c r="F17" s="8" t="n"/>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-hasSubstrate-hasMeasuredProperty-Thickness</t>
+          <t>hasNegativeElectrode-echem:hasSubstrate-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
       <c r="F18" s="4" t="n"/>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-hasSubstrate-hasMeasuredProperty-Porosity</t>
+          <t>hasNegativeElectrode-echem:hasSubstrate-hasMeasuredProperty-Porosity</t>
         </is>
       </c>
       <c r="F28" s="4" t="n"/>
@@ -1404,7 +1404,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-hasSubstrate-schema:manufacturer</t>
+          <t>hasNegativeElectrode-echem:hasSubstrate-schema:manufacturer</t>
         </is>
       </c>
       <c r="F33" s="4" t="n"/>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-hasSubstrate-schema:productID</t>
+          <t>hasNegativeElectrode-echem:hasSubstrate-schema:productID</t>
         </is>
       </c>
       <c r="F34" s="8" t="n"/>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>ImmersionElectrode</t>
+          <t>echem:ImmersionElectrode</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>hasPositiveElectrode-hasSubstrate</t>
+          <t>hasPositiveElectrode-echem:hasSubstrate</t>
         </is>
       </c>
       <c r="F41" s="12" t="n"/>
@@ -1638,7 +1638,7 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>hasPositiveElectrode-hasSubstrate</t>
+          <t>hasPositiveElectrode-echem:hasSubstrate</t>
         </is>
       </c>
       <c r="F42" s="4" t="n"/>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>hasPositiveElectrode-hasSubstrate-hasMeasuredProperty-Thickness</t>
+          <t>hasPositiveElectrode-echem:hasSubstrate-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
       <c r="F43" s="12" t="n"/>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>hasPositiveElectrode-hasSubstrate-hasMeasuredProperty-Porosity</t>
+          <t>hasPositiveElectrode-echem:hasSubstrate-hasMeasuredProperty-Porosity</t>
         </is>
       </c>
       <c r="F53" s="4" t="n"/>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>hasPositiveElectrode-hasSubstrate-schema:manufacturer</t>
+          <t>hasPositiveElectrode-echem:hasSubstrate-schema:manufacturer</t>
         </is>
       </c>
       <c r="F58" s="4" t="n"/>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="E59" s="12" t="inlineStr">
         <is>
-          <t>hasPositiveElectrode-hasSubstrate-schema:productID</t>
+          <t>hasPositiveElectrode-echem:hasSubstrate-schema:productID</t>
         </is>
       </c>
       <c r="F59" s="12" t="n"/>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-Gas</t>
+          <t>hasComponentA-type|echem:NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-Gas</t>
         </is>
       </c>
       <c r="F65" s="4" t="n"/>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="E66" s="16" t="inlineStr">
         <is>
-          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-hasMeasuredProperty-VolumeFraction</t>
+          <t>hasComponentA-type|echem:NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-hasMeasuredProperty-VolumeFraction</t>
         </is>
       </c>
       <c r="F66" s="16" t="n"/>
@@ -2270,7 +2270,7 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-Gas</t>
+          <t>hasComponentA-type|echem:NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-Gas</t>
         </is>
       </c>
       <c r="F67" s="4" t="n"/>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="E68" s="16" t="inlineStr">
         <is>
-          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-hasMeasuredProperty-VolumeFraction</t>
+          <t>hasComponentA-type|echem:NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-hasMeasuredProperty-VolumeFraction</t>
         </is>
       </c>
       <c r="F68" s="16" t="n"/>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasMeasuredProperty-VolumeFlowRate</t>
+          <t>hasComponentA-type|echem:NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasMeasuredProperty-VolumeFlowRate</t>
         </is>
       </c>
       <c r="F69" s="4" t="n"/>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="E70" s="16" t="inlineStr">
         <is>
-          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasMeasuredProperty-Pressure</t>
+          <t>hasComponentA-type|echem:NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasMeasuredProperty-Pressure</t>
         </is>
       </c>
       <c r="F70" s="16" t="n"/>
@@ -2706,7 +2706,7 @@
       </c>
       <c r="E85" s="16" t="inlineStr">
         <is>
-          <t>hasCatholyte-hasMeasuredProperty-pH</t>
+          <t>hasCatholyte-hasMeasuredProperty-PH</t>
         </is>
       </c>
       <c r="F85" s="16" t="n"/>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-Gas</t>
+          <t>hasComponentD-type|echem:PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-Gas</t>
         </is>
       </c>
       <c r="F100" s="4" t="n"/>
@@ -3090,7 +3090,7 @@
       </c>
       <c r="E101" s="16" t="inlineStr">
         <is>
-          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-hasMeasuredProperty-VolumeFraction</t>
+          <t>hasComponentD-type|echem:PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-hasMeasuredProperty-VolumeFraction</t>
         </is>
       </c>
       <c r="F101" s="16" t="n"/>
@@ -3114,7 +3114,7 @@
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-Gas</t>
+          <t>hasComponentD-type|echem:PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-Gas</t>
         </is>
       </c>
       <c r="F102" s="4" t="n"/>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="E103" s="16" t="inlineStr">
         <is>
-          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-hasMeasuredProperty-VolumeFraction</t>
+          <t>hasComponentD-type|echem:PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-hasMeasuredProperty-VolumeFraction</t>
         </is>
       </c>
       <c r="F103" s="16" t="n"/>
@@ -3164,7 +3164,7 @@
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasMeasuredProperty-VolumeFlowRate</t>
+          <t>hasComponentD-type|echem:PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasMeasuredProperty-VolumeFlowRate</t>
         </is>
       </c>
       <c r="F104" s="4" t="n"/>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="E105" s="16" t="inlineStr">
         <is>
-          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasMeasuredProperty-Pressure</t>
+          <t>hasComponentD-type|echem:PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasMeasuredProperty-Pressure</t>
         </is>
       </c>
       <c r="F105" s="16" t="n"/>
@@ -3548,7 +3548,7 @@
       </c>
       <c r="E120" s="16" t="inlineStr">
         <is>
-          <t>hasAnolyte-hasMeasuredProperty-pH</t>
+          <t>hasAnolyte-hasMeasuredProperty-PH</t>
         </is>
       </c>
       <c r="F120" s="16" t="n"/>
@@ -3975,7 +3975,7 @@
       </c>
       <c r="B138" s="5" t="inlineStr">
         <is>
-          <t>PolyArylPiperidinium</t>
+          <t>chemical:PolyArylPiperidinium</t>
         </is>
       </c>
       <c r="C138" s="5" t="inlineStr">
@@ -4404,7 +4404,7 @@
       </c>
       <c r="E155" s="5" t="inlineStr">
         <is>
-          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasComponent</t>
+          <t>hasComponentA-type|echem:NegativeElectrodeGasCompartment-hasComponent</t>
         </is>
       </c>
       <c r="F155" s="5" t="n"/>
@@ -4430,7 +4430,7 @@
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasMeasuredProperty-Width</t>
+          <t>hasComponentA-type|echem:NegativeElectrodeGasCompartment-hasMeasuredProperty-Width</t>
         </is>
       </c>
       <c r="F156" s="4" t="n"/>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasMeasuredProperty-Width</t>
+          <t>hasComponentD-type|echem:PositiveElectrodeGasCompartment-hasMeasuredProperty-Width</t>
         </is>
       </c>
       <c r="F166" s="4" t="n"/>
@@ -4722,7 +4722,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasComponent</t>
+          <t>hasComponentD-type|echem:PositiveElectrodeGasCompartment-hasComponent</t>
         </is>
       </c>
       <c r="F167" s="5" t="n"/>
@@ -5184,7 +5184,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>hasSubstrate</t>
+          <t>echem:hasSubstrate</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -5381,7 +5381,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>NegativeElectrodeGasCompartment</t>
+          <t>echem:NegativeElectrodeGasCompartment</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -5393,7 +5393,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PositiveElectrodeGasCompartment</t>
+          <t>echem:PositiveElectrodeGasCompartment</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -5420,7 +5420,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ImmersionElectrode</t>
+          <t>echem:ImmersionElectrode</t>
         </is>
       </c>
     </row>
@@ -5829,7 +5829,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>PolyArylPiperidinium</t>
+          <t>chemical:PolyArylPiperidinium</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -6191,7 +6191,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>pH</t>
+          <t>PH</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">

</xml_diff>

<commit_message>
Remove all echem prefixes
</commit_message>
<xml_diff>
--- a/test/data/electrolysis_excel_schema.xlsx
+++ b/test/data/electrolysis_excel_schema.xlsx
@@ -946,7 +946,7 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-echem:hasSubstrate</t>
+          <t>hasNegativeElectrode-hasSubstrate</t>
         </is>
       </c>
       <c r="F15" s="8" t="n"/>
@@ -974,7 +974,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-echem:hasSubstrate</t>
+          <t>hasNegativeElectrode-hasSubstrate</t>
         </is>
       </c>
       <c r="F16" s="4" t="n"/>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-echem:hasSubstrate-hasCoating</t>
+          <t>hasNegativeElectrode-hasSubstrate-hasCoating</t>
         </is>
       </c>
       <c r="F17" s="8" t="n"/>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-echem:hasSubstrate-hasMeasuredProperty-Thickness</t>
+          <t>hasNegativeElectrode-hasSubstrate-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
       <c r="F18" s="4" t="n"/>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-echem:hasSubstrate-hasMeasuredProperty-Porosity</t>
+          <t>hasNegativeElectrode-hasSubstrate-hasMeasuredProperty-Porosity</t>
         </is>
       </c>
       <c r="F28" s="4" t="n"/>
@@ -1404,7 +1404,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-echem:hasSubstrate-schema:manufacturer</t>
+          <t>hasNegativeElectrode-hasSubstrate-schema:manufacturer</t>
         </is>
       </c>
       <c r="F33" s="4" t="n"/>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>hasNegativeElectrode-echem:hasSubstrate-schema:productID</t>
+          <t>hasNegativeElectrode-hasSubstrate-schema:productID</t>
         </is>
       </c>
       <c r="F34" s="8" t="n"/>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>echem:ImmersionElectrode</t>
+          <t>ImmersionElectrode</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>hasPositiveElectrode-echem:hasSubstrate</t>
+          <t>hasPositiveElectrode-hasSubstrate</t>
         </is>
       </c>
       <c r="F41" s="12" t="n"/>
@@ -1638,7 +1638,7 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>hasPositiveElectrode-echem:hasSubstrate</t>
+          <t>hasPositiveElectrode-hasSubstrate</t>
         </is>
       </c>
       <c r="F42" s="4" t="n"/>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>hasPositiveElectrode-echem:hasSubstrate-hasMeasuredProperty-Thickness</t>
+          <t>hasPositiveElectrode-hasSubstrate-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
       <c r="F43" s="12" t="n"/>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>hasPositiveElectrode-echem:hasSubstrate-hasMeasuredProperty-Porosity</t>
+          <t>hasPositiveElectrode-hasSubstrate-hasMeasuredProperty-Porosity</t>
         </is>
       </c>
       <c r="F53" s="4" t="n"/>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>hasPositiveElectrode-echem:hasSubstrate-schema:manufacturer</t>
+          <t>hasPositiveElectrode-hasSubstrate-schema:manufacturer</t>
         </is>
       </c>
       <c r="F58" s="4" t="n"/>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="E59" s="12" t="inlineStr">
         <is>
-          <t>hasPositiveElectrode-echem:hasSubstrate-schema:productID</t>
+          <t>hasPositiveElectrode-hasSubstrate-schema:productID</t>
         </is>
       </c>
       <c r="F59" s="12" t="n"/>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>hasComponentA-type|echem:NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-Gas</t>
+          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-Gas</t>
         </is>
       </c>
       <c r="F65" s="4" t="n"/>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="E66" s="16" t="inlineStr">
         <is>
-          <t>hasComponentA-type|echem:NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-hasMeasuredProperty-VolumeFraction</t>
+          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-hasMeasuredProperty-VolumeFraction</t>
         </is>
       </c>
       <c r="F66" s="16" t="n"/>
@@ -2270,7 +2270,7 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>hasComponentA-type|echem:NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-Gas</t>
+          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-Gas</t>
         </is>
       </c>
       <c r="F67" s="4" t="n"/>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="E68" s="16" t="inlineStr">
         <is>
-          <t>hasComponentA-type|echem:NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-hasMeasuredProperty-VolumeFraction</t>
+          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-hasMeasuredProperty-VolumeFraction</t>
         </is>
       </c>
       <c r="F68" s="16" t="n"/>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>hasComponentA-type|echem:NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasMeasuredProperty-VolumeFlowRate</t>
+          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasMeasuredProperty-VolumeFlowRate</t>
         </is>
       </c>
       <c r="F69" s="4" t="n"/>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="E70" s="16" t="inlineStr">
         <is>
-          <t>hasComponentA-type|echem:NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasMeasuredProperty-Pressure</t>
+          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasMeasuredProperty-Pressure</t>
         </is>
       </c>
       <c r="F70" s="16" t="n"/>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>hasComponentD-type|echem:PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-Gas</t>
+          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-Gas</t>
         </is>
       </c>
       <c r="F100" s="4" t="n"/>
@@ -3090,7 +3090,7 @@
       </c>
       <c r="E101" s="16" t="inlineStr">
         <is>
-          <t>hasComponentD-type|echem:PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-hasMeasuredProperty-VolumeFraction</t>
+          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentA-hasMeasuredProperty-VolumeFraction</t>
         </is>
       </c>
       <c r="F101" s="16" t="n"/>
@@ -3114,7 +3114,7 @@
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>hasComponentD-type|echem:PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-Gas</t>
+          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-Gas</t>
         </is>
       </c>
       <c r="F102" s="4" t="n"/>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="E103" s="16" t="inlineStr">
         <is>
-          <t>hasComponentD-type|echem:PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-hasMeasuredProperty-VolumeFraction</t>
+          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasConstituentB-hasMeasuredProperty-VolumeFraction</t>
         </is>
       </c>
       <c r="F103" s="16" t="n"/>
@@ -3164,7 +3164,7 @@
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>hasComponentD-type|echem:PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasMeasuredProperty-VolumeFlowRate</t>
+          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasMeasuredProperty-VolumeFlowRate</t>
         </is>
       </c>
       <c r="F104" s="4" t="n"/>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="E105" s="16" t="inlineStr">
         <is>
-          <t>hasComponentD-type|echem:PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasMeasuredProperty-Pressure</t>
+          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasActiveMaterial-type|GasMixture-hasMeasuredProperty-Pressure</t>
         </is>
       </c>
       <c r="F105" s="16" t="n"/>
@@ -4404,7 +4404,7 @@
       </c>
       <c r="E155" s="5" t="inlineStr">
         <is>
-          <t>hasComponentA-type|echem:NegativeElectrodeGasCompartment-hasComponent</t>
+          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasComponent</t>
         </is>
       </c>
       <c r="F155" s="5" t="n"/>
@@ -4430,7 +4430,7 @@
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>hasComponentA-type|echem:NegativeElectrodeGasCompartment-hasMeasuredProperty-Width</t>
+          <t>hasComponentA-type|NegativeElectrodeGasCompartment-hasMeasuredProperty-Width</t>
         </is>
       </c>
       <c r="F156" s="4" t="n"/>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>hasComponentD-type|echem:PositiveElectrodeGasCompartment-hasMeasuredProperty-Width</t>
+          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasMeasuredProperty-Width</t>
         </is>
       </c>
       <c r="F166" s="4" t="n"/>
@@ -4722,7 +4722,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t>hasComponentD-type|echem:PositiveElectrodeGasCompartment-hasComponent</t>
+          <t>hasComponentD-type|PositiveElectrodeGasCompartment-hasComponent</t>
         </is>
       </c>
       <c r="F167" s="5" t="n"/>
@@ -5184,7 +5184,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>echem:hasSubstrate</t>
+          <t>hasSubstrate</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -5381,7 +5381,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>echem:NegativeElectrodeGasCompartment</t>
+          <t>NegativeElectrodeGasCompartment</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -5393,7 +5393,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>echem:PositiveElectrodeGasCompartment</t>
+          <t>PositiveElectrodeGasCompartment</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -5420,7 +5420,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>echem:ImmersionElectrode</t>
+          <t>ImmersionElectrode</t>
         </is>
       </c>
     </row>

</xml_diff>